<commit_message>
Weekly NBA competitor report 2026-08-18
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor Ranking" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30-Day Growth" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Posting Activity" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Competitor Ranking" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="30-Day Growth" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Posting Activity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Issues" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="History" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$L$43</definedName>
@@ -358,14 +358,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -390,10 +390,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="00B8D9"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="00B8D9"/>
               </a:solidFill>
@@ -427,8 +427,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -454,8 +454,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -478,14 +478,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -509,10 +509,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="12B76A"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="12B76A"/>
               </a:solidFill>
@@ -546,8 +546,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -573,8 +573,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -597,7 +597,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -612,9 +612,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -634,9 +634,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>56491</v>
+        <v>56490</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>17775</v>
+        <v>17776</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="I19" s="17" t="n">
         <v>0.7</v>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>56491</v>
+        <v>56490</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17775</v>
+        <v>17776</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2002,10 +2002,10 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>56491</v>
+        <v>56490</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E2" s="29" t="n">
         <v>0.7</v>
@@ -2018,7 +2018,9 @@
       <c r="G2" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H2" s="27" t="n"/>
+      <c r="H2" s="27" t="n">
+        <v>7718</v>
+      </c>
       <c r="I2" s="28" t="n"/>
       <c r="J2" s="26" t="inlineStr">
         <is>
@@ -2072,13 +2074,13 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>17775</v>
+        <v>17776</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2088,7 +2090,9 @@
       <c r="G4" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="H4" s="27" t="n"/>
+      <c r="H4" s="27" t="n">
+        <v>6775</v>
+      </c>
       <c r="I4" s="28" t="n"/>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2159,7 +2163,7 @@
         <v>35</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>2956</v>
+        <v>2955</v>
       </c>
       <c r="I6" s="28" t="n"/>
       <c r="J6" s="26" t="inlineStr">
@@ -2178,10 +2182,10 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15362</v>
+        <v>15363</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E7" s="29" t="n">
         <v>0.0107</v>
@@ -2286,13 +2290,13 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>10974</v>
+        <v>10973</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>-26</v>
+        <v>-27</v>
       </c>
       <c r="E10" s="30" t="n">
-        <v>-0.24</v>
+        <v>-0.25</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -2466,13 +2470,13 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4639</v>
+        <v>4638</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>-61</v>
+        <v>-62</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>-0.013</v>
+        <v>-0.0132</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -2943,13 +2947,13 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>56491</v>
+        <v>56490</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>56100</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E5" s="29" t="n">
         <v>0.7</v>
@@ -3033,16 +3037,16 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>17775</v>
+        <v>17776</v>
       </c>
       <c r="C8" s="27" t="n">
         <v>17700</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -3243,13 +3247,13 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>15362</v>
+        <v>15363</v>
       </c>
       <c r="C15" s="27" t="n">
         <v>15200</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E15" s="29" t="n">
         <v>0.0107</v>
@@ -3273,16 +3277,16 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>4639</v>
+        <v>4638</v>
       </c>
       <c r="C16" s="27" t="n">
         <v>4700</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-61</v>
+        <v>-62</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.013</v>
+        <v>-0.0132</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -3423,16 +3427,16 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>10974</v>
+        <v>10973</v>
       </c>
       <c r="C21" s="27" t="n">
         <v>11000</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-26</v>
+        <v>-27</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.24</v>
+        <v>-0.25</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -3554,7 +3558,9 @@
           <t>ifbbproleagueoz</t>
         </is>
       </c>
-      <c r="B2" s="27" t="n"/>
+      <c r="B2" s="27" t="n">
+        <v>7718</v>
+      </c>
       <c r="C2" s="28" t="n"/>
       <c r="D2" s="26" t="inlineStr"/>
     </row>
@@ -3576,7 +3582,9 @@
           <t>icnqld</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n"/>
+      <c r="B4" s="27" t="n">
+        <v>6775</v>
+      </c>
       <c r="C4" s="28" t="n"/>
       <c r="D4" s="26" t="inlineStr"/>
     </row>
@@ -3599,7 +3607,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>2956</v>
+        <v>2955</v>
       </c>
       <c r="C6" s="28" t="n"/>
       <c r="D6" s="26" t="inlineStr"/>
@@ -9646,7 +9654,7 @@
         </is>
       </c>
       <c r="C288" s="27" t="n">
-        <v>10974</v>
+        <v>10973</v>
       </c>
       <c r="D288" s="26" t="inlineStr">
         <is>
@@ -9706,7 +9714,7 @@
         </is>
       </c>
       <c r="C291" s="27" t="n">
-        <v>56491</v>
+        <v>56490</v>
       </c>
       <c r="D291" s="26" t="inlineStr">
         <is>
@@ -9726,7 +9734,7 @@
         </is>
       </c>
       <c r="C292" s="27" t="n">
-        <v>15362</v>
+        <v>15363</v>
       </c>
       <c r="D292" s="26" t="inlineStr">
         <is>
@@ -9866,7 +9874,7 @@
         </is>
       </c>
       <c r="C299" s="27" t="n">
-        <v>4639</v>
+        <v>4638</v>
       </c>
       <c r="D299" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-08-23
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 18 August 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 23 August 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,308</t>
+          <t>18,320</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+59.00%</t>
+          <t>+66.00%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+108 followers • 35 days</t>
+          <t>+120 followers • 40 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,25 +1261,25 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>56490</v>
+        <v>56503</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>@anb.australia</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>40d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,25 +1295,25 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18308</v>
+        <v>18320</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@icn_nsw</t>
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>13</v>
+        <v>143</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>40d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>17776</v>
+        <v>17786</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
@@ -1340,14 +1340,14 @@
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>40d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,25 +1363,25 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>15884</v>
+        <v>15943</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>@ifbbproleagueoz</t>
+          <t>@anb.australia</t>
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>390</v>
+        <v>80</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.7</v>
+        <v>0.84</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>40d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,25 +1397,25 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15878</v>
+        <v>15836</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>@nbaaustralia_official</t>
+          <t>@ifbbproleagueoz</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>108</v>
+        <v>403</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.59</v>
+        <v>0.72</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>35d</t>
+          <t>40d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,15 +1808,15 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>56490</v>
+        <v>56503</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>@anb.australia</t>
+          <t>@icn_nt</t>
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,15 +1826,15 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18308</v>
+        <v>18320</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>@icn_nt</t>
+          <t>@icn_nsw</t>
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17776</v>
+        <v>17786</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,15 +1862,15 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>15884</v>
+        <v>15943</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>@ifbbproleagueoz</t>
+          <t>@anb.australia</t>
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.7</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,15 +1880,15 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15878</v>
+        <v>15836</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>@nbaaustralia_official</t>
+          <t>@ifbbproleagueoz</t>
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.59</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,13 +2002,13 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>56490</v>
+        <v>56503</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>390</v>
+        <v>403</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
@@ -2016,12 +2016,14 @@
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H2" s="27" t="n">
-        <v>7718</v>
-      </c>
-      <c r="I2" s="28" t="n"/>
+        <v>7723</v>
+      </c>
+      <c r="I2" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="J2" s="26" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2038,13 +2040,13 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18308</v>
+        <v>18320</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.59</v>
+        <v>0.66</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
@@ -2052,12 +2054,14 @@
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3288</v>
-      </c>
-      <c r="I3" s="28" t="n"/>
+        <v>3292</v>
+      </c>
+      <c r="I3" s="28" t="n">
+        <v>4</v>
+      </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2074,13 +2078,13 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>17776</v>
+        <v>17786</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.43</v>
+        <v>0.49</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2088,12 +2092,14 @@
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6775</v>
-      </c>
-      <c r="I4" s="28" t="n"/>
+        <v>6780</v>
+      </c>
+      <c r="I4" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2110,13 +2116,13 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>15884</v>
+        <v>15943</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>84</v>
+        <v>143</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.53</v>
+        <v>0.91</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
@@ -2124,12 +2130,14 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>6751</v>
-      </c>
-      <c r="I5" s="28" t="n"/>
+        <v>6758</v>
+      </c>
+      <c r="I5" s="28" t="n">
+        <v>7</v>
+      </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2146,13 +2154,13 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15878</v>
+        <v>15836</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>-22</v>
+        <v>-64</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>-0.14</v>
+        <v>-0.4</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -2160,12 +2168,14 @@
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>2955</v>
-      </c>
-      <c r="I6" s="28" t="n"/>
+        <v>2960</v>
+      </c>
+      <c r="I6" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2182,13 +2192,13 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15363</v>
+        <v>15391</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>163</v>
+        <v>191</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0107</v>
+        <v>0.0126</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
@@ -2196,12 +2206,14 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3562</v>
-      </c>
-      <c r="I7" s="28" t="n"/>
+        <v>3569</v>
+      </c>
+      <c r="I7" s="28" t="n">
+        <v>7</v>
+      </c>
       <c r="J7" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2218,13 +2230,13 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>12683</v>
+        <v>12723</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>-17</v>
-      </c>
-      <c r="E8" s="30" t="n">
-        <v>-0.13</v>
+        <v>23</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>0.18</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -2232,12 +2244,14 @@
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4459</v>
-      </c>
-      <c r="I8" s="28" t="n"/>
+        <v>4461</v>
+      </c>
+      <c r="I8" s="28" t="n">
+        <v>2</v>
+      </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2254,13 +2268,13 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11394</v>
+        <v>11403</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
@@ -2268,12 +2282,14 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2825</v>
-      </c>
-      <c r="I9" s="28" t="n"/>
+        <v>2830</v>
+      </c>
+      <c r="I9" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2304,12 +2320,14 @@
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H10" s="27" t="n">
-        <v>4368</v>
-      </c>
-      <c r="I10" s="28" t="n"/>
+        <v>4370</v>
+      </c>
+      <c r="I10" s="28" t="n">
+        <v>2</v>
+      </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2326,13 +2344,13 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9589</v>
+        <v>9580</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.84</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
@@ -2340,12 +2358,14 @@
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2717</v>
-      </c>
-      <c r="I11" s="28" t="n"/>
+        <v>2725</v>
+      </c>
+      <c r="I11" s="28" t="n">
+        <v>8</v>
+      </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2362,13 +2382,13 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7190</v>
+        <v>7204</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0127</v>
+        <v>0.0146</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -2376,12 +2396,14 @@
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>819</v>
-      </c>
-      <c r="I12" s="28" t="n"/>
+        <v>823</v>
+      </c>
+      <c r="I12" s="28" t="n">
+        <v>4</v>
+      </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2412,12 +2434,14 @@
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3100</v>
-      </c>
-      <c r="I13" s="28" t="n"/>
+        <v>3104</v>
+      </c>
+      <c r="I13" s="28" t="n">
+        <v>4</v>
+      </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2434,13 +2458,13 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6434</v>
+        <v>6495</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>134</v>
+        <v>195</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0213</v>
+        <v>0.031</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
@@ -2448,12 +2472,14 @@
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1086</v>
-      </c>
-      <c r="I14" s="28" t="n"/>
+        <v>1093</v>
+      </c>
+      <c r="I14" s="28" t="n">
+        <v>7</v>
+      </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2470,13 +2496,13 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4638</v>
+        <v>4635</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>-62</v>
+        <v>-65</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>-0.0132</v>
+        <v>-0.0138</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -2484,12 +2510,14 @@
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H15" s="27" t="n">
         <v>815</v>
       </c>
-      <c r="I15" s="28" t="n"/>
+      <c r="I15" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="J15" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2506,13 +2534,13 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4581</v>
+        <v>4583</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-19</v>
+        <v>-17</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.41</v>
+        <v>-0.37</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -2520,12 +2548,14 @@
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H16" s="27" t="n">
-        <v>1870</v>
-      </c>
-      <c r="I16" s="28" t="n"/>
+        <v>1872</v>
+      </c>
+      <c r="I16" s="28" t="n">
+        <v>2</v>
+      </c>
       <c r="J16" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2542,13 +2572,13 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2277</v>
+        <v>2278</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>-1</v>
+        <v>-0.96</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
@@ -2556,12 +2586,14 @@
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>2145</v>
-      </c>
-      <c r="I17" s="28" t="n"/>
+        <v>2146</v>
+      </c>
+      <c r="I17" s="28" t="n">
+        <v>1</v>
+      </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2578,13 +2610,13 @@
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>2125</v>
+        <v>2159</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.0119</v>
+        <v>0.0281</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
@@ -2592,12 +2624,14 @@
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H18" s="27" t="n">
         <v>331</v>
       </c>
-      <c r="I18" s="28" t="n"/>
+      <c r="I18" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="J18" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2614,13 +2648,13 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1836</v>
+        <v>1839</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.02</v>
+        <v>0.0217</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
@@ -2628,12 +2662,14 @@
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H19" s="27" t="n">
-        <v>175</v>
-      </c>
-      <c r="I19" s="28" t="n"/>
+        <v>176</v>
+      </c>
+      <c r="I19" s="28" t="n">
+        <v>1</v>
+      </c>
       <c r="J19" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2650,13 +2686,13 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1830</v>
+        <v>1833</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0167</v>
+        <v>0.0183</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
@@ -2664,12 +2700,14 @@
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>208</v>
-      </c>
-      <c r="I20" s="28" t="n"/>
+        <v>210</v>
+      </c>
+      <c r="I20" s="28" t="n">
+        <v>2</v>
+      </c>
       <c r="J20" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2686,13 +2724,13 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1448</v>
+        <v>1446</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-52</v>
+        <v>-54</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.0347</v>
+        <v>-0.036</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -2700,12 +2738,14 @@
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H21" s="27" t="n">
         <v>1357</v>
       </c>
-      <c r="I21" s="28" t="n"/>
+      <c r="I21" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="J21" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2736,12 +2776,14 @@
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H22" s="27" t="n">
-        <v>297</v>
-      </c>
-      <c r="I22" s="28" t="n"/>
+        <v>298</v>
+      </c>
+      <c r="I22" s="28" t="n">
+        <v>1</v>
+      </c>
       <c r="J22" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2758,13 +2800,13 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.0246</v>
+        <v>0.0302</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
@@ -2772,12 +2814,14 @@
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>628</v>
-      </c>
-      <c r="I23" s="28" t="n"/>
+        <v>636</v>
+      </c>
+      <c r="I23" s="28" t="n">
+        <v>8</v>
+      </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2853,20 +2897,20 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>anb.australia</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>9589</v>
+        <v>1413</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>9500</v>
+        <v>1400</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
@@ -2874,29 +2918,29 @@
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H2" s="26" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>icn_nsw</t>
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>1413</v>
+        <v>15943</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>1400</v>
+        <v>15800</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>13</v>
+        <v>143</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
@@ -2904,10 +2948,10 @@
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H3" s="26" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" ht="21" customHeight="1">
@@ -2917,16 +2961,16 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>11394</v>
+        <v>11403</v>
       </c>
       <c r="C4" s="27" t="n">
         <v>11300</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2934,7 +2978,7 @@
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H4" s="26" t="n">
         <v>8</v>
@@ -2943,20 +2987,20 @@
     <row r="5" ht="21" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>anb.australia</t>
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>56490</v>
+        <v>9580</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>56100</v>
+        <v>9500</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>390</v>
+        <v>80</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.7</v>
+        <v>0.84</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
@@ -2964,29 +3008,29 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>nbaaustralia_official</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>18308</v>
+        <v>56503</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>18200</v>
+        <v>56100</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>108</v>
+        <v>403</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.59</v>
+        <v>0.72</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -2994,29 +3038,29 @@
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>icn_nsw</t>
+          <t>nbaaustralia_official</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>15884</v>
+        <v>18320</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15800</v>
+        <v>18200</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
@@ -3024,10 +3068,10 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
@@ -3037,16 +3081,16 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>17776</v>
+        <v>17786</v>
       </c>
       <c r="C8" s="27" t="n">
         <v>17700</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.43</v>
+        <v>0.49</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -3054,7 +3098,7 @@
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H8" s="26" t="n">
         <v>3</v>
@@ -3063,20 +3107,20 @@
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_vic</t>
+          <t>icn_victoria</t>
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>915</v>
+        <v>12723</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>893</v>
+        <v>12700</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0246</v>
+        <v>0.18</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
@@ -3084,10 +3128,10 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
@@ -3097,16 +3141,16 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>6434</v>
+        <v>6495</v>
       </c>
       <c r="C10" s="27" t="n">
         <v>6300</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>134</v>
+        <v>195</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0213</v>
+        <v>0.031</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -3114,7 +3158,7 @@
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H10" s="26" t="n">
         <v>13</v>
@@ -3123,20 +3167,20 @@
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>icn.indonesia</t>
+          <t>msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>1836</v>
+        <v>920</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>1800</v>
+        <v>893</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.02</v>
+        <v>0.0302</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
@@ -3144,29 +3188,29 @@
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>cbrfitexpo</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>1830</v>
+        <v>2159</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>1800</v>
+        <v>2100</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0167</v>
+        <v>0.0281</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -3174,29 +3218,29 @@
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>wnbfaustralia</t>
+          <t>icn.indonesia</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>7190</v>
+        <v>1839</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>7100</v>
+        <v>1800</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>90</v>
+        <v>39</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0127</v>
+        <v>0.0217</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
@@ -3204,29 +3248,29 @@
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>cbrfitexpo</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>2125</v>
+        <v>1833</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>2100</v>
+        <v>1800</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0119</v>
+        <v>0.0183</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
@@ -3234,29 +3278,29 @@
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia</t>
+          <t>wnbfaustralia</t>
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>15363</v>
+        <v>7204</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>15200</v>
+        <v>7100</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>163</v>
+        <v>104</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0107</v>
+        <v>0.0146</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -3264,29 +3308,29 @@
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H15" s="26" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>ynf_australia</t>
+          <t>msfitnessaustralia</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>4638</v>
+        <v>15391</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4700</v>
+        <v>15200</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-62</v>
-      </c>
-      <c r="E16" s="30" t="n">
-        <v>-0.0132</v>
+        <v>191</v>
+      </c>
+      <c r="E16" s="29" t="n">
+        <v>0.0126</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -3294,29 +3338,29 @@
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H16" s="26" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_perth</t>
+          <t>ynf_australia</t>
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>1448</v>
+        <v>4635</v>
       </c>
       <c r="C17" s="27" t="n">
-        <v>1500</v>
+        <v>4700</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>-52</v>
+        <v>-65</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>-0.0347</v>
+        <v>-0.0138</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
@@ -3324,29 +3368,29 @@
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H17" s="26" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>icn_sa</t>
+          <t>msfitnessaustralia_perth</t>
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>6697</v>
+        <v>1446</v>
       </c>
       <c r="C18" s="27" t="n">
-        <v>6700</v>
+        <v>1500</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>-3</v>
+        <v>-54</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>-0.04</v>
+        <v>-0.036</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
@@ -3354,29 +3398,29 @@
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>icn_victoria</t>
+          <t>icn_sa</t>
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>12683</v>
+        <v>6697</v>
       </c>
       <c r="C19" s="27" t="n">
-        <v>12700</v>
+        <v>6700</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>-17</v>
+        <v>-3</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>-0.13</v>
+        <v>-0.04</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
@@ -3384,29 +3428,29 @@
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>nabbaaustralia</t>
+          <t>icn_wa</t>
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>15878</v>
+        <v>10973</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>15900</v>
+        <v>11000</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>-22</v>
+        <v>-27</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>-0.14</v>
+        <v>-0.25</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
@@ -3414,29 +3458,29 @@
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H20" s="26" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>icn_wa</t>
+          <t>icn_act</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>10973</v>
+        <v>4583</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>11000</v>
+        <v>4600</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-27</v>
+        <v>-17</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.25</v>
+        <v>-0.37</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -3444,29 +3488,29 @@
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H21" s="26" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>icn_act</t>
+          <t>nabbaaustralia</t>
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>4581</v>
+        <v>15836</v>
       </c>
       <c r="C22" s="27" t="n">
-        <v>4600</v>
+        <v>15900</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-19</v>
+        <v>-64</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.41</v>
+        <v>-0.4</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
@@ -3474,10 +3518,10 @@
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H22" s="26" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" ht="21" customHeight="1">
@@ -3487,16 +3531,16 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>2277</v>
+        <v>2278</v>
       </c>
       <c r="C23" s="27" t="n">
         <v>2300</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>-1</v>
+        <v>-0.96</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
@@ -3504,7 +3548,7 @@
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H23" s="26" t="n">
         <v>16</v>
@@ -3559,10 +3603,16 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>7718</v>
-      </c>
-      <c r="C2" s="28" t="n"/>
-      <c r="D2" s="26" t="inlineStr"/>
+        <v>7723</v>
+      </c>
+      <c r="C2" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
@@ -3571,10 +3621,16 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3288</v>
-      </c>
-      <c r="C3" s="28" t="n"/>
-      <c r="D3" s="26" t="inlineStr"/>
+        <v>3292</v>
+      </c>
+      <c r="C3" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
@@ -3583,10 +3639,16 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6775</v>
-      </c>
-      <c r="C4" s="28" t="n"/>
-      <c r="D4" s="26" t="inlineStr"/>
+        <v>6780</v>
+      </c>
+      <c r="C4" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="21" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
@@ -3595,10 +3657,16 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6751</v>
-      </c>
-      <c r="C5" s="28" t="n"/>
-      <c r="D5" s="26" t="inlineStr"/>
+        <v>6758</v>
+      </c>
+      <c r="C5" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
@@ -3607,10 +3675,16 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>2955</v>
-      </c>
-      <c r="C6" s="28" t="n"/>
-      <c r="D6" s="26" t="inlineStr"/>
+        <v>2960</v>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
@@ -3619,10 +3693,16 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3562</v>
-      </c>
-      <c r="C7" s="28" t="n"/>
-      <c r="D7" s="26" t="inlineStr"/>
+        <v>3569</v>
+      </c>
+      <c r="C7" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
@@ -3631,10 +3711,16 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4459</v>
-      </c>
-      <c r="C8" s="28" t="n"/>
-      <c r="D8" s="26" t="inlineStr"/>
+        <v>4461</v>
+      </c>
+      <c r="C8" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
@@ -3643,10 +3729,16 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2825</v>
-      </c>
-      <c r="C9" s="28" t="n"/>
-      <c r="D9" s="26" t="inlineStr"/>
+        <v>2830</v>
+      </c>
+      <c r="C9" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
@@ -3655,10 +3747,16 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4368</v>
-      </c>
-      <c r="C10" s="28" t="n"/>
-      <c r="D10" s="26" t="inlineStr"/>
+        <v>4370</v>
+      </c>
+      <c r="C10" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
@@ -3667,10 +3765,16 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2717</v>
-      </c>
-      <c r="C11" s="28" t="n"/>
-      <c r="D11" s="26" t="inlineStr"/>
+        <v>2725</v>
+      </c>
+      <c r="C11" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
@@ -3679,10 +3783,16 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>819</v>
-      </c>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="26" t="inlineStr"/>
+        <v>823</v>
+      </c>
+      <c r="C12" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
@@ -3691,10 +3801,16 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3100</v>
-      </c>
-      <c r="C13" s="28" t="n"/>
-      <c r="D13" s="26" t="inlineStr"/>
+        <v>3104</v>
+      </c>
+      <c r="C13" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
@@ -3703,10 +3819,16 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1086</v>
-      </c>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="26" t="inlineStr"/>
+        <v>1093</v>
+      </c>
+      <c r="C14" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
@@ -3717,8 +3839,14 @@
       <c r="B15" s="27" t="n">
         <v>815</v>
       </c>
-      <c r="C15" s="28" t="n"/>
-      <c r="D15" s="26" t="inlineStr"/>
+      <c r="C15" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
@@ -3727,10 +3855,16 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>1870</v>
-      </c>
-      <c r="C16" s="28" t="n"/>
-      <c r="D16" s="26" t="inlineStr"/>
+        <v>1872</v>
+      </c>
+      <c r="C16" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="21" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
@@ -3739,10 +3873,16 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>2145</v>
-      </c>
-      <c r="C17" s="28" t="n"/>
-      <c r="D17" s="26" t="inlineStr"/>
+        <v>2146</v>
+      </c>
+      <c r="C17" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="21" customHeight="1">
       <c r="A18" s="26" t="inlineStr">
@@ -3753,8 +3893,14 @@
       <c r="B18" s="27" t="n">
         <v>331</v>
       </c>
-      <c r="C18" s="28" t="n"/>
-      <c r="D18" s="26" t="inlineStr"/>
+      <c r="C18" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
@@ -3763,10 +3909,16 @@
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>175</v>
-      </c>
-      <c r="C19" s="28" t="n"/>
-      <c r="D19" s="26" t="inlineStr"/>
+        <v>176</v>
+      </c>
+      <c r="C19" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
@@ -3775,10 +3927,16 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>208</v>
-      </c>
-      <c r="C20" s="28" t="n"/>
-      <c r="D20" s="26" t="inlineStr"/>
+        <v>210</v>
+      </c>
+      <c r="C20" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
@@ -3789,8 +3947,14 @@
       <c r="B21" s="27" t="n">
         <v>1357</v>
       </c>
-      <c r="C21" s="28" t="n"/>
-      <c r="D21" s="26" t="inlineStr"/>
+      <c r="C21" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="21" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
@@ -3799,10 +3963,16 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>297</v>
-      </c>
-      <c r="C22" s="28" t="n"/>
-      <c r="D22" s="26" t="inlineStr"/>
+        <v>298</v>
+      </c>
+      <c r="C22" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="21" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
@@ -3811,10 +3981,16 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>628</v>
-      </c>
-      <c r="C23" s="28" t="n"/>
-      <c r="D23" s="26" t="inlineStr"/>
+        <v>636</v>
+      </c>
+      <c r="C23" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3861,7 +4037,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -3891,7 +4067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D299"/>
+  <dimension ref="A1:D321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9882,6 +10058,446 @@
         </is>
       </c>
     </row>
+    <row r="300" ht="21" customHeight="1">
+      <c r="A300" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B300" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C300" s="27" t="n">
+        <v>9580</v>
+      </c>
+      <c r="D300" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="21" customHeight="1">
+      <c r="A301" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B301" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C301" s="27" t="n">
+        <v>2159</v>
+      </c>
+      <c r="D301" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="21" customHeight="1">
+      <c r="A302" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B302" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C302" s="27" t="n">
+        <v>1833</v>
+      </c>
+      <c r="D302" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="21" customHeight="1">
+      <c r="A303" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B303" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C303" s="27" t="n">
+        <v>1839</v>
+      </c>
+      <c r="D303" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="21" customHeight="1">
+      <c r="A304" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B304" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C304" s="27" t="n">
+        <v>4583</v>
+      </c>
+      <c r="D304" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="21" customHeight="1">
+      <c r="A305" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B305" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C305" s="27" t="n">
+        <v>15943</v>
+      </c>
+      <c r="D305" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="21" customHeight="1">
+      <c r="A306" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B306" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C306" s="27" t="n">
+        <v>1413</v>
+      </c>
+      <c r="D306" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="21" customHeight="1">
+      <c r="A307" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B307" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C307" s="27" t="n">
+        <v>6697</v>
+      </c>
+      <c r="D307" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="21" customHeight="1">
+      <c r="A308" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B308" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C308" s="27" t="n">
+        <v>2278</v>
+      </c>
+      <c r="D308" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="21" customHeight="1">
+      <c r="A309" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B309" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C309" s="27" t="n">
+        <v>12723</v>
+      </c>
+      <c r="D309" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="21" customHeight="1">
+      <c r="A310" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B310" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C310" s="27" t="n">
+        <v>10973</v>
+      </c>
+      <c r="D310" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="21" customHeight="1">
+      <c r="A311" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B311" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C311" s="27" t="n">
+        <v>6495</v>
+      </c>
+      <c r="D311" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="21" customHeight="1">
+      <c r="A312" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B312" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C312" s="27" t="n">
+        <v>17786</v>
+      </c>
+      <c r="D312" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="21" customHeight="1">
+      <c r="A313" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B313" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C313" s="27" t="n">
+        <v>56503</v>
+      </c>
+      <c r="D313" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="21" customHeight="1">
+      <c r="A314" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B314" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C314" s="27" t="n">
+        <v>15391</v>
+      </c>
+      <c r="D314" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="21" customHeight="1">
+      <c r="A315" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B315" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C315" s="27" t="n">
+        <v>1446</v>
+      </c>
+      <c r="D315" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="21" customHeight="1">
+      <c r="A316" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B316" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C316" s="27" t="n">
+        <v>920</v>
+      </c>
+      <c r="D316" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="21" customHeight="1">
+      <c r="A317" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B317" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C317" s="27" t="n">
+        <v>15836</v>
+      </c>
+      <c r="D317" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="21" customHeight="1">
+      <c r="A318" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B318" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C318" s="27" t="n">
+        <v>18320</v>
+      </c>
+      <c r="D318" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="21" customHeight="1">
+      <c r="A319" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B319" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C319" s="27" t="n">
+        <v>11403</v>
+      </c>
+      <c r="D319" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="21" customHeight="1">
+      <c r="A320" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B320" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C320" s="27" t="n">
+        <v>7204</v>
+      </c>
+      <c r="D320" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="321" ht="21" customHeight="1">
+      <c r="A321" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B321" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C321" s="27" t="n">
+        <v>4635</v>
+      </c>
+      <c r="D321" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-08-31
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 23 August 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 31 August 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,320</t>
+          <t>18,339</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+0.66%</t>
+          <t>+0.76%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+120 followers • 40 days</t>
+          <t>+139 followers • 48 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,25 +1261,25 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>56503</v>
+        <v>56838</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>@icnnewzealand</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>195</v>
+        <v>34</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.031</v>
+        <v>0.0381</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>40d</t>
+          <t>48d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,25 +1295,25 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18320</v>
+        <v>18339</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@cbrfitexpo</t>
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.0302</v>
+        <v>0.0348</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>40d</t>
+          <t>48d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,25 +1329,25 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>17787</v>
+        <v>17793</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>@cbrfitexpo</t>
+          <t>@icnnewzealand</t>
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>58</v>
+        <v>198</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.0276</v>
+        <v>0.0314</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>40d</t>
+          <t>48d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>15943</v>
+        <v>16017</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
@@ -1374,14 +1374,14 @@
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0217</v>
+        <v>0.0239</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>40d</t>
+          <t>48d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,25 +1397,25 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15836</v>
+        <v>15793</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="14" t="inlineStr">
         <is>
-          <t>@dfba_global</t>
+          <t>@anb.australia</t>
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>33</v>
+        <v>217</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.0183</v>
+        <v>0.0228</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>40d</t>
+          <t>48d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,15 +1808,15 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>56503</v>
+        <v>56838</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>@icnnewzealand</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.031</v>
+        <v>0.0381</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,15 +1826,15 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18320</v>
+        <v>18339</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@cbrfitexpo</t>
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.0302</v>
+        <v>0.0348</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,15 +1844,15 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17787</v>
+        <v>17793</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>@cbrfitexpo</t>
+          <t>@icnnewzealand</t>
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.0276</v>
+        <v>0.0314</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>15943</v>
+        <v>16017</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0217</v>
+        <v>0.0239</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,15 +1880,15 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15836</v>
+        <v>15793</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>@dfba_global</t>
+          <t>@anb.australia</t>
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.0183</v>
+        <v>0.0228</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,13 +2002,13 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>56503</v>
+        <v>56838</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>403</v>
+        <v>738</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0072</v>
+        <v>0.0132</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
@@ -2016,13 +2016,13 @@
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H2" s="27" t="n">
-        <v>7723</v>
+        <v>7802</v>
       </c>
       <c r="I2" s="28" t="n">
-        <v>5</v>
+        <v>79</v>
       </c>
       <c r="J2" s="26" t="inlineStr">
         <is>
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18320</v>
+        <v>18339</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0066</v>
+        <v>0.0076</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
@@ -2054,13 +2054,13 @@
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3292</v>
+        <v>3299</v>
       </c>
       <c r="I3" s="28" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
@@ -2078,13 +2078,13 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>17787</v>
+        <v>17793</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0049</v>
+        <v>0.0053</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2092,13 +2092,13 @@
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6780</v>
+        <v>6784</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2116,13 +2116,13 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>15943</v>
+        <v>16017</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>143</v>
+        <v>217</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0091</v>
+        <v>0.0137</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
@@ -2130,13 +2130,13 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>6758</v>
+        <v>6764</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
@@ -2154,13 +2154,13 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15836</v>
+        <v>15793</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>-64</v>
+        <v>-107</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>-0.004</v>
+        <v>-0.0067</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -2168,13 +2168,13 @@
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>2960</v>
+        <v>2963</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
@@ -2192,13 +2192,13 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15391</v>
+        <v>15440</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>191</v>
+        <v>240</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0126</v>
+        <v>0.0158</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
@@ -2206,13 +2206,13 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3569</v>
+        <v>3579</v>
       </c>
       <c r="I7" s="28" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J7" s="26" t="inlineStr">
         <is>
@@ -2230,13 +2230,13 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>12723</v>
+        <v>12801</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>23</v>
+        <v>101</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0018</v>
+        <v>0.008</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -2244,13 +2244,13 @@
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H8" s="27" t="n">
         <v>4461</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
@@ -2268,13 +2268,13 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11403</v>
+        <v>11410</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0091</v>
+        <v>0.0097</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
@@ -2282,13 +2282,13 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2830</v>
+        <v>2836</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,13 +2306,13 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>10973</v>
+        <v>10978</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>-27</v>
+        <v>-22</v>
       </c>
       <c r="E10" s="30" t="n">
-        <v>-0.0025</v>
+        <v>-0.002</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -2320,13 +2320,13 @@
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H10" s="27" t="n">
         <v>4370</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
@@ -2344,13 +2344,13 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9580</v>
+        <v>9717</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>80</v>
+        <v>217</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.0228</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
@@ -2358,13 +2358,13 @@
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2725</v>
+        <v>2734</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
@@ -2382,13 +2382,13 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7204</v>
+        <v>7211</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0146</v>
+        <v>0.0156</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -2396,13 +2396,13 @@
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>823</v>
+        <v>829</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
@@ -2420,13 +2420,13 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6697</v>
+        <v>6709</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>-3</v>
-      </c>
-      <c r="E13" s="30" t="n">
-        <v>-0.0004</v>
+        <v>9</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>0.0013</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
@@ -2434,13 +2434,13 @@
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3104</v>
+        <v>3106</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,13 +2458,13 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6495</v>
+        <v>6498</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.031</v>
+        <v>0.0314</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
@@ -2472,14 +2472,12 @@
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1093</v>
-      </c>
-      <c r="I14" s="28" t="n">
-        <v>7</v>
-      </c>
+        <v>1087</v>
+      </c>
+      <c r="I14" s="28" t="n"/>
       <c r="J14" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2496,13 +2494,13 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4635</v>
+        <v>4629</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>-65</v>
+        <v>-71</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>-0.0138</v>
+        <v>-0.0151</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -2510,7 +2508,7 @@
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H15" s="27" t="n">
         <v>815</v>
@@ -2534,13 +2532,13 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4583</v>
+        <v>4588</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-17</v>
+        <v>-12</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.0037</v>
+        <v>-0.0026</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -2548,13 +2546,13 @@
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H16" s="27" t="n">
-        <v>1872</v>
+        <v>1876</v>
       </c>
       <c r="I16" s="28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J16" s="26" t="inlineStr">
         <is>
@@ -2572,13 +2570,13 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2278</v>
+        <v>2276</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-0.0104</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
@@ -2586,13 +2584,13 @@
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>2146</v>
+        <v>2148</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -2610,13 +2608,13 @@
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>2158</v>
+        <v>2173</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.0276</v>
+        <v>0.0348</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
@@ -2624,13 +2622,13 @@
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H18" s="27" t="n">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="I18" s="28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J18" s="26" t="inlineStr">
         <is>
@@ -2648,13 +2646,13 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1839</v>
+        <v>1843</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0217</v>
+        <v>0.0239</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
@@ -2662,13 +2660,13 @@
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H19" s="27" t="n">
         <v>176</v>
       </c>
       <c r="I19" s="28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" s="26" t="inlineStr">
         <is>
@@ -2686,13 +2684,13 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1833</v>
+        <v>1829</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0183</v>
+        <v>0.0161</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
@@ -2700,10 +2698,10 @@
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I20" s="28" t="n">
         <v>2</v>
@@ -2724,13 +2722,13 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1446</v>
+        <v>1444</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-54</v>
+        <v>-56</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.036</v>
+        <v>-0.0373</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -2738,7 +2736,7 @@
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H21" s="27" t="n">
         <v>1357</v>
@@ -2762,13 +2760,13 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E22" s="29" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
@@ -2776,13 +2774,13 @@
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H22" s="27" t="n">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J22" s="26" t="inlineStr">
         <is>
@@ -2800,13 +2798,13 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>920</v>
+        <v>927</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.0302</v>
+        <v>0.0381</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
@@ -2814,13 +2812,13 @@
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>636</v>
+        <v>648</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
@@ -2897,20 +2895,20 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>icnnewzealand</t>
+          <t>msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>6495</v>
+        <v>927</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>6300</v>
+        <v>893</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>195</v>
+        <v>34</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.031</v>
+        <v>0.0381</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
@@ -2918,29 +2916,29 @@
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H2" s="26" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_vic</t>
+          <t>cbrfitexpo</t>
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>920</v>
+        <v>2173</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>893</v>
+        <v>2100</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0302</v>
+        <v>0.0348</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
@@ -2948,29 +2946,29 @@
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H3" s="26" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" ht="21" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>cbrfitexpo</t>
+          <t>icnnewzealand</t>
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>2158</v>
+        <v>6498</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>2100</v>
+        <v>6300</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>58</v>
+        <v>198</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0276</v>
+        <v>0.0314</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2978,10 +2976,10 @@
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H4" s="26" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" ht="21" customHeight="1">
@@ -2991,16 +2989,16 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>1839</v>
+        <v>1843</v>
       </c>
       <c r="C5" s="27" t="n">
         <v>1800</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0217</v>
+        <v>0.0239</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
@@ -3008,7 +3006,7 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H5" s="26" t="n">
         <v>18</v>
@@ -3017,20 +3015,20 @@
     <row r="6" ht="21" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>anb.australia</t>
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>1833</v>
+        <v>9717</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>1800</v>
+        <v>9500</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>33</v>
+        <v>217</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0183</v>
+        <v>0.0228</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -3038,29 +3036,29 @@
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H6" s="26" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>wnbfaustralia</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>7204</v>
+        <v>1829</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>7100</v>
+        <v>1800</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>104</v>
+        <v>29</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0146</v>
+        <v>0.0161</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
@@ -3068,10 +3066,10 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
@@ -3081,16 +3079,16 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>15391</v>
+        <v>15440</v>
       </c>
       <c r="C8" s="27" t="n">
         <v>15200</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>191</v>
+        <v>240</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0126</v>
+        <v>0.0158</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -3098,7 +3096,7 @@
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H8" s="26" t="n">
         <v>6</v>
@@ -3107,20 +3105,20 @@
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>wnbfaustralia</t>
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>1413</v>
+        <v>7211</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>1400</v>
+        <v>7100</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>13</v>
+        <v>111</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.0156</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
@@ -3128,10 +3126,10 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
@@ -3141,16 +3139,16 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>15943</v>
+        <v>16017</v>
       </c>
       <c r="C10" s="27" t="n">
         <v>15800</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>143</v>
+        <v>217</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0091</v>
+        <v>0.0137</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -3158,7 +3156,7 @@
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H10" s="26" t="n">
         <v>4</v>
@@ -3167,20 +3165,20 @@
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>pca_australia</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>11403</v>
+        <v>56838</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>11300</v>
+        <v>56100</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>103</v>
+        <v>738</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0091</v>
+        <v>0.0132</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
@@ -3188,29 +3186,29 @@
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>anb.australia</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>9580</v>
+        <v>1414</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>9500</v>
+        <v>1400</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -3218,29 +3216,29 @@
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>pca_australia</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>56503</v>
+        <v>11410</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>56100</v>
+        <v>11300</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>403</v>
+        <v>110</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0072</v>
+        <v>0.0097</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
@@ -3248,29 +3246,29 @@
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>nbaaustralia_official</t>
+          <t>icn_victoria</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>18320</v>
+        <v>12801</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>18200</v>
+        <v>12700</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0066</v>
+        <v>0.008</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
@@ -3278,29 +3276,29 @@
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>icnqld</t>
+          <t>nbaaustralia_official</t>
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>17787</v>
+        <v>18339</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>17700</v>
+        <v>18200</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>87</v>
+        <v>139</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0049</v>
+        <v>0.0076</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -3308,29 +3306,29 @@
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H15" s="26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>icn_victoria</t>
+          <t>icnqld</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>12723</v>
+        <v>17793</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>12700</v>
+        <v>17700</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.0018</v>
+        <v>0.0053</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -3338,10 +3336,10 @@
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H16" s="26" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
@@ -3351,16 +3349,16 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>6697</v>
+        <v>6709</v>
       </c>
       <c r="C17" s="27" t="n">
         <v>6700</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>-3</v>
-      </c>
-      <c r="E17" s="30" t="n">
-        <v>-0.0004</v>
+        <v>9</v>
+      </c>
+      <c r="E17" s="29" t="n">
+        <v>0.0013</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
@@ -3368,7 +3366,7 @@
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H17" s="26" t="n">
         <v>12</v>
@@ -3381,16 +3379,16 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>10973</v>
+        <v>10978</v>
       </c>
       <c r="C18" s="27" t="n">
         <v>11000</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>-27</v>
+        <v>-22</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>-0.0025</v>
+        <v>-0.002</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
@@ -3398,7 +3396,7 @@
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H18" s="26" t="n">
         <v>9</v>
@@ -3411,16 +3409,16 @@
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>4583</v>
+        <v>4588</v>
       </c>
       <c r="C19" s="27" t="n">
         <v>4600</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>-17</v>
+        <v>-12</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>-0.0037</v>
+        <v>-0.0026</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
@@ -3428,7 +3426,7 @@
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H19" s="26" t="n">
         <v>15</v>
@@ -3441,16 +3439,16 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>15836</v>
+        <v>15793</v>
       </c>
       <c r="C20" s="27" t="n">
         <v>15900</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>-64</v>
+        <v>-107</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>-0.004</v>
+        <v>-0.0067</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
@@ -3458,7 +3456,7 @@
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H20" s="26" t="n">
         <v>5</v>
@@ -3471,16 +3469,16 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>2278</v>
+        <v>2276</v>
       </c>
       <c r="C21" s="27" t="n">
         <v>2300</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-22</v>
+        <v>-24</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.009599999999999999</v>
+        <v>-0.0104</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -3488,7 +3486,7 @@
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H21" s="26" t="n">
         <v>16</v>
@@ -3501,16 +3499,16 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>4635</v>
+        <v>4629</v>
       </c>
       <c r="C22" s="27" t="n">
         <v>4700</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-65</v>
+        <v>-71</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0138</v>
+        <v>-0.0151</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
@@ -3518,7 +3516,7 @@
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H22" s="26" t="n">
         <v>14</v>
@@ -3531,16 +3529,16 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>1446</v>
+        <v>1444</v>
       </c>
       <c r="C23" s="27" t="n">
         <v>1500</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-54</v>
+        <v>-56</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>-0.036</v>
+        <v>-0.0373</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
@@ -3548,7 +3546,7 @@
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H23" s="26" t="n">
         <v>20</v>
@@ -3603,14 +3601,14 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>7723</v>
+        <v>7802</v>
       </c>
       <c r="C2" s="28" t="n">
-        <v>5</v>
+        <v>79</v>
       </c>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3621,14 +3619,14 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3292</v>
+        <v>3299</v>
       </c>
       <c r="C3" s="28" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3639,14 +3637,14 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6780</v>
+        <v>6784</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3657,14 +3655,14 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6758</v>
+        <v>6764</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3675,14 +3673,14 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>2960</v>
+        <v>2963</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3693,14 +3691,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3569</v>
+        <v>3579</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3714,11 +3712,11 @@
         <v>4461</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3729,14 +3727,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2830</v>
+        <v>2836</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3750,11 +3748,11 @@
         <v>4370</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3765,14 +3763,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2725</v>
+        <v>2734</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3783,14 +3781,14 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>823</v>
+        <v>829</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3801,14 +3799,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3104</v>
+        <v>3106</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3819,14 +3817,12 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1093</v>
-      </c>
-      <c r="C14" s="28" t="n">
-        <v>7</v>
-      </c>
+        <v>1087</v>
+      </c>
+      <c r="C14" s="28" t="n"/>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3840,7 @@
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3855,14 +3851,14 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>1872</v>
+        <v>1876</v>
       </c>
       <c r="C16" s="28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3873,14 +3869,14 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>2146</v>
+        <v>2148</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3891,14 +3887,14 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C18" s="28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3912,11 +3908,11 @@
         <v>176</v>
       </c>
       <c r="C19" s="28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3927,14 +3923,14 @@
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C20" s="28" t="n">
         <v>2</v>
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3952,7 +3948,7 @@
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3963,14 +3959,14 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C22" s="28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -3981,14 +3977,14 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>636</v>
+        <v>648</v>
       </c>
       <c r="C23" s="28" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4033,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4067,7 +4063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D321"/>
+  <dimension ref="A1:D343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10498,6 +10494,446 @@
         </is>
       </c>
     </row>
+    <row r="322" ht="21" customHeight="1">
+      <c r="A322" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B322" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C322" s="27" t="n">
+        <v>9717</v>
+      </c>
+      <c r="D322" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="21" customHeight="1">
+      <c r="A323" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B323" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C323" s="27" t="n">
+        <v>2173</v>
+      </c>
+      <c r="D323" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" ht="21" customHeight="1">
+      <c r="A324" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B324" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C324" s="27" t="n">
+        <v>1829</v>
+      </c>
+      <c r="D324" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="21" customHeight="1">
+      <c r="A325" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B325" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C325" s="27" t="n">
+        <v>1843</v>
+      </c>
+      <c r="D325" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" ht="21" customHeight="1">
+      <c r="A326" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B326" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C326" s="27" t="n">
+        <v>4588</v>
+      </c>
+      <c r="D326" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="327" ht="21" customHeight="1">
+      <c r="A327" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B327" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C327" s="27" t="n">
+        <v>16017</v>
+      </c>
+      <c r="D327" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="21" customHeight="1">
+      <c r="A328" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B328" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C328" s="27" t="n">
+        <v>1414</v>
+      </c>
+      <c r="D328" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="21" customHeight="1">
+      <c r="A329" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B329" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C329" s="27" t="n">
+        <v>6709</v>
+      </c>
+      <c r="D329" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="21" customHeight="1">
+      <c r="A330" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B330" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C330" s="27" t="n">
+        <v>2276</v>
+      </c>
+      <c r="D330" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="331" ht="21" customHeight="1">
+      <c r="A331" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B331" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C331" s="27" t="n">
+        <v>12801</v>
+      </c>
+      <c r="D331" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="21" customHeight="1">
+      <c r="A332" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B332" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C332" s="27" t="n">
+        <v>10978</v>
+      </c>
+      <c r="D332" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="21" customHeight="1">
+      <c r="A333" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B333" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C333" s="27" t="n">
+        <v>6498</v>
+      </c>
+      <c r="D333" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="334" ht="21" customHeight="1">
+      <c r="A334" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B334" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C334" s="27" t="n">
+        <v>17793</v>
+      </c>
+      <c r="D334" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="21" customHeight="1">
+      <c r="A335" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B335" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C335" s="27" t="n">
+        <v>56838</v>
+      </c>
+      <c r="D335" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="336" ht="21" customHeight="1">
+      <c r="A336" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B336" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C336" s="27" t="n">
+        <v>15440</v>
+      </c>
+      <c r="D336" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="21" customHeight="1">
+      <c r="A337" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B337" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C337" s="27" t="n">
+        <v>1444</v>
+      </c>
+      <c r="D337" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="21" customHeight="1">
+      <c r="A338" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B338" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C338" s="27" t="n">
+        <v>927</v>
+      </c>
+      <c r="D338" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="21" customHeight="1">
+      <c r="A339" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B339" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C339" s="27" t="n">
+        <v>15793</v>
+      </c>
+      <c r="D339" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="21" customHeight="1">
+      <c r="A340" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B340" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C340" s="27" t="n">
+        <v>18339</v>
+      </c>
+      <c r="D340" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="21" customHeight="1">
+      <c r="A341" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B341" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C341" s="27" t="n">
+        <v>11410</v>
+      </c>
+      <c r="D341" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="342" ht="21" customHeight="1">
+      <c r="A342" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B342" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C342" s="27" t="n">
+        <v>7211</v>
+      </c>
+      <c r="D342" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="21" customHeight="1">
+      <c r="A343" s="26" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B343" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C343" s="27" t="n">
+        <v>4629</v>
+      </c>
+      <c r="D343" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly NBA competitor report 2026-09-06
</commit_message>
<xml_diff>
--- a/data/NBA_Competitor_Report_Latest.xlsx
+++ b/data/NBA_Competitor_Report_Latest.xlsx
@@ -1000,7 +1000,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Instagram competitor growth • 31 August 2026 • 30-day+ comparison</t>
+          <t>Instagram competitor growth • 06 September 2026 • 30-day+ comparison</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>18,339</t>
+          <t>18,425</t>
         </is>
       </c>
       <c r="B8" s="7" t="n"/>
@@ -1090,7 +1090,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>+0.76%</t>
+          <t>+1.24%</t>
         </is>
       </c>
       <c r="H8" s="7" t="n"/>
@@ -1146,7 +1146,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>+139 followers • 48 days</t>
+          <t>+225 followers • 54 days</t>
         </is>
       </c>
       <c r="H11" s="7" t="n"/>
@@ -1261,25 +1261,25 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>56838</v>
+        <v>57539</v>
       </c>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@cbrfitexpo</t>
         </is>
       </c>
       <c r="H16" s="16" t="n">
-        <v>34</v>
+        <v>120</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>0.0381</v>
+        <v>0.0571</v>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>48d</t>
+          <t>54d</t>
         </is>
       </c>
       <c r="K16" s="5" t="n"/>
@@ -1295,25 +1295,25 @@
         </is>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18339</v>
+        <v>18425</v>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>@cbrfitexpo</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H17" s="16" t="n">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>0.0348</v>
+        <v>0.047</v>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>48d</t>
+          <t>54d</t>
         </is>
       </c>
       <c r="K17" s="5" t="n"/>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="C18" s="15" t="n">
-        <v>17793</v>
+        <v>17835</v>
       </c>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
@@ -1340,14 +1340,14 @@
         </is>
       </c>
       <c r="H18" s="16" t="n">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>0.0314</v>
+        <v>0.0344</v>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>48d</t>
+          <t>54d</t>
         </is>
       </c>
       <c r="K18" s="5" t="n"/>
@@ -1363,25 +1363,25 @@
         </is>
       </c>
       <c r="C19" s="15" t="n">
-        <v>16017</v>
+        <v>16036</v>
       </c>
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>@icn.indonesia</t>
+          <t>@ifbbproleagueoz</t>
         </is>
       </c>
       <c r="H19" s="16" t="n">
-        <v>43</v>
+        <v>1439</v>
       </c>
       <c r="I19" s="17" t="n">
-        <v>0.0239</v>
+        <v>0.0257</v>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>48d</t>
+          <t>54d</t>
         </is>
       </c>
       <c r="K19" s="5" t="n"/>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="C20" s="15" t="n">
-        <v>15793</v>
+        <v>15721</v>
       </c>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
@@ -1408,14 +1408,14 @@
         </is>
       </c>
       <c r="H20" s="16" t="n">
-        <v>217</v>
+        <v>234</v>
       </c>
       <c r="I20" s="17" t="n">
-        <v>0.0228</v>
+        <v>0.0246</v>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>48d</t>
+          <t>54d</t>
         </is>
       </c>
       <c r="K20" s="5" t="n"/>
@@ -1808,15 +1808,15 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>56838</v>
+        <v>57539</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>@msfitnessaustralia_vic</t>
+          <t>@cbrfitexpo</t>
         </is>
       </c>
       <c r="H48" s="24" t="n">
-        <v>0.0381</v>
+        <v>0.0571</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -1826,15 +1826,15 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>18339</v>
+        <v>18425</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>@cbrfitexpo</t>
+          <t>@msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="H49" s="24" t="n">
-        <v>0.0348</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17793</v>
+        <v>17835</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         </is>
       </c>
       <c r="H50" s="24" t="n">
-        <v>0.0314</v>
+        <v>0.0344</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -1862,15 +1862,15 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16017</v>
+        <v>16036</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>@icn.indonesia</t>
+          <t>@ifbbproleagueoz</t>
         </is>
       </c>
       <c r="H51" s="24" t="n">
-        <v>0.0239</v>
+        <v>0.0257</v>
       </c>
     </row>
     <row r="52" hidden="1">
@@ -1880,7 +1880,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15793</v>
+        <v>15721</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="H52" s="24" t="n">
-        <v>0.0228</v>
+        <v>0.0246</v>
       </c>
     </row>
     <row r="53" hidden="1"/>
@@ -2002,13 +2002,13 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>56838</v>
+        <v>57539</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>738</v>
+        <v>1439</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0132</v>
+        <v>0.0257</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
@@ -2016,13 +2016,13 @@
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H2" s="27" t="n">
-        <v>7802</v>
+        <v>7970</v>
       </c>
       <c r="I2" s="28" t="n">
-        <v>79</v>
+        <v>168</v>
       </c>
       <c r="J2" s="26" t="inlineStr">
         <is>
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="C3" s="27" t="n">
-        <v>18339</v>
+        <v>18425</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>139</v>
+        <v>225</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0076</v>
+        <v>0.0124</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
@@ -2054,13 +2054,13 @@
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H3" s="27" t="n">
-        <v>3299</v>
+        <v>3335</v>
       </c>
       <c r="I3" s="28" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
@@ -2078,13 +2078,13 @@
         </is>
       </c>
       <c r="C4" s="27" t="n">
-        <v>17793</v>
+        <v>17835</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>93</v>
+        <v>135</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0053</v>
+        <v>0.0076</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2092,13 +2092,13 @@
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H4" s="27" t="n">
-        <v>6784</v>
+        <v>6786</v>
       </c>
       <c r="I4" s="28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
@@ -2116,13 +2116,13 @@
         </is>
       </c>
       <c r="C5" s="27" t="n">
-        <v>16017</v>
+        <v>16036</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0137</v>
+        <v>0.0149</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
@@ -2130,13 +2130,13 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H5" s="27" t="n">
-        <v>6764</v>
+        <v>6786</v>
       </c>
       <c r="I5" s="28" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
@@ -2154,13 +2154,13 @@
         </is>
       </c>
       <c r="C6" s="27" t="n">
-        <v>15793</v>
+        <v>15721</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>-107</v>
+        <v>-179</v>
       </c>
       <c r="E6" s="30" t="n">
-        <v>-0.0067</v>
+        <v>-0.0113</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -2168,13 +2168,13 @@
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H6" s="27" t="n">
-        <v>2963</v>
+        <v>2970</v>
       </c>
       <c r="I6" s="28" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J6" s="26" t="inlineStr">
         <is>
@@ -2192,13 +2192,13 @@
         </is>
       </c>
       <c r="C7" s="27" t="n">
-        <v>15440</v>
+        <v>15466</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>240</v>
+        <v>266</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0158</v>
+        <v>0.0175</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
@@ -2206,10 +2206,10 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>3579</v>
+        <v>3589</v>
       </c>
       <c r="I7" s="28" t="n">
         <v>10</v>
@@ -2230,13 +2230,13 @@
         </is>
       </c>
       <c r="C8" s="27" t="n">
-        <v>12801</v>
+        <v>12893</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>101</v>
+        <v>193</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.008</v>
+        <v>0.0152</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -2244,13 +2244,13 @@
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>4461</v>
+        <v>4462</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
@@ -2268,13 +2268,13 @@
         </is>
       </c>
       <c r="C9" s="27" t="n">
-        <v>11410</v>
+        <v>11413</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0097</v>
+        <v>0.01</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
@@ -2282,13 +2282,13 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>2836</v>
+        <v>2846</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
@@ -2306,13 +2306,13 @@
         </is>
       </c>
       <c r="C10" s="27" t="n">
-        <v>10978</v>
+        <v>10997</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>-22</v>
+        <v>-3</v>
       </c>
       <c r="E10" s="30" t="n">
-        <v>-0.002</v>
+        <v>-0.0003</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -2320,13 +2320,13 @@
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H10" s="27" t="n">
-        <v>4370</v>
+        <v>4373</v>
       </c>
       <c r="I10" s="28" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J10" s="26" t="inlineStr">
         <is>
@@ -2344,13 +2344,13 @@
         </is>
       </c>
       <c r="C11" s="27" t="n">
-        <v>9717</v>
+        <v>9734</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>217</v>
+        <v>234</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0228</v>
+        <v>0.0246</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
@@ -2358,13 +2358,13 @@
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>2734</v>
+        <v>2741</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J11" s="26" t="inlineStr">
         <is>
@@ -2382,13 +2382,13 @@
         </is>
       </c>
       <c r="C12" s="27" t="n">
-        <v>7211</v>
+        <v>7252</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>111</v>
+        <v>152</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.0156</v>
+        <v>0.0214</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -2396,13 +2396,13 @@
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H12" s="27" t="n">
-        <v>829</v>
+        <v>832</v>
       </c>
       <c r="I12" s="28" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J12" s="26" t="inlineStr">
         <is>
@@ -2420,13 +2420,13 @@
         </is>
       </c>
       <c r="C13" s="27" t="n">
-        <v>6709</v>
+        <v>6716</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0013</v>
+        <v>0.0024</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
@@ -2434,13 +2434,13 @@
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>3106</v>
+        <v>3114</v>
       </c>
       <c r="I13" s="28" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J13" s="26" t="inlineStr">
         <is>
@@ -2458,13 +2458,13 @@
         </is>
       </c>
       <c r="C14" s="27" t="n">
-        <v>6498</v>
+        <v>6517</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.0314</v>
+        <v>0.0344</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
@@ -2472,12 +2472,14 @@
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>1087</v>
-      </c>
-      <c r="I14" s="28" t="n"/>
+        <v>1093</v>
+      </c>
+      <c r="I14" s="28" t="n">
+        <v>6</v>
+      </c>
       <c r="J14" s="26" t="inlineStr">
         <is>
           <t>no</t>
@@ -2494,13 +2496,13 @@
         </is>
       </c>
       <c r="C15" s="27" t="n">
-        <v>4629</v>
+        <v>4620</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>-71</v>
+        <v>-80</v>
       </c>
       <c r="E15" s="30" t="n">
-        <v>-0.0151</v>
+        <v>-0.017</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -2508,7 +2510,7 @@
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H15" s="27" t="n">
         <v>815</v>
@@ -2532,13 +2534,13 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>4588</v>
+        <v>4591</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="E16" s="30" t="n">
-        <v>-0.0026</v>
+        <v>-0.002</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -2546,13 +2548,13 @@
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H16" s="27" t="n">
-        <v>1876</v>
+        <v>1884</v>
       </c>
       <c r="I16" s="28" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J16" s="26" t="inlineStr">
         <is>
@@ -2570,13 +2572,13 @@
         </is>
       </c>
       <c r="C17" s="27" t="n">
-        <v>2276</v>
+        <v>2277</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="E17" s="30" t="n">
-        <v>-0.0104</v>
+        <v>-0.01</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
@@ -2584,13 +2586,13 @@
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H17" s="27" t="n">
-        <v>2148</v>
+        <v>2149</v>
       </c>
       <c r="I17" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" s="26" t="inlineStr">
         <is>
@@ -2608,13 +2610,13 @@
         </is>
       </c>
       <c r="C18" s="27" t="n">
-        <v>2173</v>
+        <v>2220</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>0.0348</v>
+        <v>0.0571</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
@@ -2622,10 +2624,10 @@
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H18" s="27" t="n">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="I18" s="28" t="n">
         <v>2</v>
@@ -2646,13 +2648,13 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1843</v>
+        <v>1838</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.0239</v>
+        <v>0.0211</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
@@ -2660,7 +2662,7 @@
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H19" s="27" t="n">
         <v>176</v>
@@ -2684,13 +2686,13 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1829</v>
+        <v>1837</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>0.0161</v>
+        <v>0.0206</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
@@ -2698,13 +2700,13 @@
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H20" s="27" t="n">
         <v>212</v>
       </c>
       <c r="I20" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J20" s="26" t="inlineStr">
         <is>
@@ -2722,13 +2724,13 @@
         </is>
       </c>
       <c r="C21" s="27" t="n">
-        <v>1444</v>
+        <v>1442</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-56</v>
+        <v>-58</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.0373</v>
+        <v>-0.0387</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -2736,7 +2738,7 @@
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H21" s="27" t="n">
         <v>1357</v>
@@ -2760,13 +2762,13 @@
         </is>
       </c>
       <c r="C22" s="27" t="n">
-        <v>1414</v>
+        <v>1432</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="E22" s="29" t="n">
-        <v>0.01</v>
+        <v>0.0229</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
@@ -2774,13 +2776,13 @@
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H22" s="27" t="n">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="I22" s="28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J22" s="26" t="inlineStr">
         <is>
@@ -2798,13 +2800,13 @@
         </is>
       </c>
       <c r="C23" s="27" t="n">
-        <v>927</v>
+        <v>935</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.0381</v>
+        <v>0.047</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
@@ -2812,13 +2814,13 @@
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H23" s="27" t="n">
-        <v>648</v>
+        <v>662</v>
       </c>
       <c r="I23" s="28" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J23" s="26" t="inlineStr">
         <is>
@@ -2895,20 +2897,20 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia_vic</t>
+          <t>cbrfitexpo</t>
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>927</v>
+        <v>2220</v>
       </c>
       <c r="C2" s="27" t="n">
-        <v>893</v>
+        <v>2100</v>
       </c>
       <c r="D2" s="28" t="n">
-        <v>34</v>
+        <v>120</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>0.0381</v>
+        <v>0.0571</v>
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
@@ -2916,29 +2918,29 @@
         </is>
       </c>
       <c r="G2" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H2" s="26" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" ht="21" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
-          <t>cbrfitexpo</t>
+          <t>msfitnessaustralia_vic</t>
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>2173</v>
+        <v>935</v>
       </c>
       <c r="C3" s="27" t="n">
-        <v>2100</v>
+        <v>893</v>
       </c>
       <c r="D3" s="28" t="n">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>0.0348</v>
+        <v>0.047</v>
       </c>
       <c r="F3" s="26" t="inlineStr">
         <is>
@@ -2946,10 +2948,10 @@
         </is>
       </c>
       <c r="G3" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H3" s="26" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" ht="21" customHeight="1">
@@ -2959,16 +2961,16 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6498</v>
+        <v>6517</v>
       </c>
       <c r="C4" s="27" t="n">
         <v>6300</v>
       </c>
       <c r="D4" s="28" t="n">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>0.0314</v>
+        <v>0.0344</v>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -2976,7 +2978,7 @@
         </is>
       </c>
       <c r="G4" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H4" s="26" t="n">
         <v>13</v>
@@ -2985,20 +2987,20 @@
     <row r="5" ht="21" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>icn.indonesia</t>
+          <t>ifbbproleagueoz</t>
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>1843</v>
+        <v>57539</v>
       </c>
       <c r="C5" s="27" t="n">
-        <v>1800</v>
+        <v>56100</v>
       </c>
       <c r="D5" s="28" t="n">
-        <v>43</v>
+        <v>1439</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.0239</v>
+        <v>0.0257</v>
       </c>
       <c r="F5" s="26" t="inlineStr">
         <is>
@@ -3006,10 +3008,10 @@
         </is>
       </c>
       <c r="G5" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H5" s="26" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="21" customHeight="1">
@@ -3019,16 +3021,16 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>9717</v>
+        <v>9734</v>
       </c>
       <c r="C6" s="27" t="n">
         <v>9500</v>
       </c>
       <c r="D6" s="28" t="n">
-        <v>217</v>
+        <v>234</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>0.0228</v>
+        <v>0.0246</v>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -3036,7 +3038,7 @@
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H6" s="26" t="n">
         <v>10</v>
@@ -3045,20 +3047,20 @@
     <row r="7" ht="21" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
-          <t>dfba_global</t>
+          <t>icn_nt</t>
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>1829</v>
+        <v>1432</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>1800</v>
+        <v>1400</v>
       </c>
       <c r="D7" s="28" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.0161</v>
+        <v>0.0229</v>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
@@ -3066,29 +3068,29 @@
         </is>
       </c>
       <c r="G7" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>msfitnessaustralia</t>
+          <t>wnbfaustralia</t>
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>15440</v>
+        <v>7252</v>
       </c>
       <c r="C8" s="27" t="n">
-        <v>15200</v>
+        <v>7100</v>
       </c>
       <c r="D8" s="28" t="n">
-        <v>240</v>
+        <v>152</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.0158</v>
+        <v>0.0214</v>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -3096,29 +3098,29 @@
         </is>
       </c>
       <c r="G8" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H8" s="26" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>wnbfaustralia</t>
+          <t>icn.indonesia</t>
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>7211</v>
+        <v>1838</v>
       </c>
       <c r="C9" s="27" t="n">
-        <v>7100</v>
+        <v>1800</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>111</v>
+        <v>38</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.0156</v>
+        <v>0.0211</v>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
@@ -3126,29 +3128,29 @@
         </is>
       </c>
       <c r="G9" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>icn_nsw</t>
+          <t>dfba_global</t>
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>16017</v>
+        <v>1837</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>15800</v>
+        <v>1800</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>217</v>
+        <v>37</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>0.0137</v>
+        <v>0.0206</v>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -3156,29 +3158,29 @@
         </is>
       </c>
       <c r="G10" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>ifbbproleagueoz</t>
+          <t>msfitnessaustralia</t>
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>56838</v>
+        <v>15466</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>56100</v>
+        <v>15200</v>
       </c>
       <c r="D11" s="28" t="n">
-        <v>738</v>
+        <v>266</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.0132</v>
+        <v>0.0175</v>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
@@ -3186,29 +3188,29 @@
         </is>
       </c>
       <c r="G11" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>icn_nt</t>
+          <t>icn_victoria</t>
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>1414</v>
+        <v>12893</v>
       </c>
       <c r="C12" s="27" t="n">
-        <v>1400</v>
+        <v>12700</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>14</v>
+        <v>193</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>0.01</v>
+        <v>0.0152</v>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -3216,29 +3218,29 @@
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H12" s="26" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>pca_australia</t>
+          <t>icn_nsw</t>
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>11410</v>
+        <v>16036</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>11300</v>
+        <v>15800</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>110</v>
+        <v>236</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.0097</v>
+        <v>0.0149</v>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
@@ -3246,29 +3248,29 @@
         </is>
       </c>
       <c r="G13" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H13" s="26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>icn_victoria</t>
+          <t>nbaaustralia_official</t>
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>12801</v>
+        <v>18425</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>12700</v>
+        <v>18200</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>101</v>
+        <v>225</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>0.008</v>
+        <v>0.0124</v>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
@@ -3276,29 +3278,29 @@
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H14" s="26" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>nbaaustralia_official</t>
+          <t>pca_australia</t>
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>18339</v>
+        <v>11413</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>18200</v>
+        <v>11300</v>
       </c>
       <c r="D15" s="28" t="n">
-        <v>139</v>
+        <v>113</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.0076</v>
+        <v>0.01</v>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
@@ -3306,10 +3308,10 @@
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H15" s="26" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
@@ -3319,16 +3321,16 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>17793</v>
+        <v>17835</v>
       </c>
       <c r="C16" s="27" t="n">
         <v>17700</v>
       </c>
       <c r="D16" s="28" t="n">
-        <v>93</v>
+        <v>135</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.0053</v>
+        <v>0.0076</v>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
@@ -3336,7 +3338,7 @@
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H16" s="26" t="n">
         <v>3</v>
@@ -3349,16 +3351,16 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>6709</v>
+        <v>6716</v>
       </c>
       <c r="C17" s="27" t="n">
         <v>6700</v>
       </c>
       <c r="D17" s="28" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.0013</v>
+        <v>0.0024</v>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
@@ -3366,7 +3368,7 @@
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H17" s="26" t="n">
         <v>12</v>
@@ -3379,16 +3381,16 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>10978</v>
+        <v>10997</v>
       </c>
       <c r="C18" s="27" t="n">
         <v>11000</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>-22</v>
+        <v>-3</v>
       </c>
       <c r="E18" s="30" t="n">
-        <v>-0.002</v>
+        <v>-0.0003</v>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
@@ -3396,7 +3398,7 @@
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H18" s="26" t="n">
         <v>9</v>
@@ -3409,16 +3411,16 @@
         </is>
       </c>
       <c r="B19" s="27" t="n">
-        <v>4588</v>
+        <v>4591</v>
       </c>
       <c r="C19" s="27" t="n">
         <v>4600</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="E19" s="30" t="n">
-        <v>-0.0026</v>
+        <v>-0.002</v>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
@@ -3426,7 +3428,7 @@
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H19" s="26" t="n">
         <v>15</v>
@@ -3435,20 +3437,20 @@
     <row r="20" ht="21" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t>nabbaaustralia</t>
+          <t>icn_tasmania</t>
         </is>
       </c>
       <c r="B20" s="27" t="n">
-        <v>15793</v>
+        <v>2277</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>15900</v>
+        <v>2300</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>-107</v>
+        <v>-23</v>
       </c>
       <c r="E20" s="30" t="n">
-        <v>-0.0067</v>
+        <v>-0.01</v>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
@@ -3456,29 +3458,29 @@
         </is>
       </c>
       <c r="G20" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H20" s="26" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>icn_tasmania</t>
+          <t>nabbaaustralia</t>
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>2276</v>
+        <v>15721</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>2300</v>
+        <v>15900</v>
       </c>
       <c r="D21" s="28" t="n">
-        <v>-24</v>
+        <v>-179</v>
       </c>
       <c r="E21" s="30" t="n">
-        <v>-0.0104</v>
+        <v>-0.0113</v>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
@@ -3486,10 +3488,10 @@
         </is>
       </c>
       <c r="G21" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H21" s="26" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
@@ -3499,16 +3501,16 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>4629</v>
+        <v>4620</v>
       </c>
       <c r="C22" s="27" t="n">
         <v>4700</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>-71</v>
+        <v>-80</v>
       </c>
       <c r="E22" s="30" t="n">
-        <v>-0.0151</v>
+        <v>-0.017</v>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
@@ -3516,7 +3518,7 @@
         </is>
       </c>
       <c r="G22" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H22" s="26" t="n">
         <v>14</v>
@@ -3529,16 +3531,16 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>1444</v>
+        <v>1442</v>
       </c>
       <c r="C23" s="27" t="n">
         <v>1500</v>
       </c>
       <c r="D23" s="28" t="n">
-        <v>-56</v>
+        <v>-58</v>
       </c>
       <c r="E23" s="30" t="n">
-        <v>-0.0373</v>
+        <v>-0.0387</v>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
@@ -3546,7 +3548,7 @@
         </is>
       </c>
       <c r="G23" s="26" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H23" s="26" t="n">
         <v>20</v>
@@ -3601,14 +3603,14 @@
         </is>
       </c>
       <c r="B2" s="27" t="n">
-        <v>7802</v>
+        <v>7970</v>
       </c>
       <c r="C2" s="28" t="n">
-        <v>79</v>
+        <v>168</v>
       </c>
       <c r="D2" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3619,14 +3621,14 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>3299</v>
+        <v>3335</v>
       </c>
       <c r="C3" s="28" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="D3" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3637,14 +3639,14 @@
         </is>
       </c>
       <c r="B4" s="27" t="n">
-        <v>6784</v>
+        <v>6786</v>
       </c>
       <c r="C4" s="28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D4" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3655,14 +3657,14 @@
         </is>
       </c>
       <c r="B5" s="27" t="n">
-        <v>6764</v>
+        <v>6786</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D5" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3673,14 +3675,14 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>2963</v>
+        <v>2970</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3691,14 +3693,14 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>3579</v>
+        <v>3589</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>10</v>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3709,14 +3711,14 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>4461</v>
+        <v>4462</v>
       </c>
       <c r="C8" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3727,14 +3729,14 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>2836</v>
+        <v>2846</v>
       </c>
       <c r="C9" s="28" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3745,14 +3747,14 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>4370</v>
+        <v>4373</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3763,14 +3765,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2734</v>
+        <v>2741</v>
       </c>
       <c r="C11" s="28" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3781,14 +3783,14 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>829</v>
+        <v>832</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3799,14 +3801,14 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>3106</v>
+        <v>3114</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3817,12 +3819,14 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>1087</v>
-      </c>
-      <c r="C14" s="28" t="n"/>
+        <v>1093</v>
+      </c>
+      <c r="C14" s="28" t="n">
+        <v>6</v>
+      </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3844,7 @@
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3851,14 +3855,14 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>1876</v>
+        <v>1884</v>
       </c>
       <c r="C16" s="28" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3869,14 +3873,14 @@
         </is>
       </c>
       <c r="B17" s="27" t="n">
-        <v>2148</v>
+        <v>2149</v>
       </c>
       <c r="C17" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3887,14 +3891,14 @@
         </is>
       </c>
       <c r="B18" s="27" t="n">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C18" s="28" t="n">
         <v>2</v>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3916,7 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3926,11 +3930,11 @@
         <v>212</v>
       </c>
       <c r="C20" s="28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3948,7 +3952,7 @@
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3959,14 +3963,14 @@
         </is>
       </c>
       <c r="B22" s="27" t="n">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="C22" s="28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3977,14 +3981,14 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>648</v>
+        <v>662</v>
       </c>
       <c r="C23" s="28" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4037,7 @@
     <row r="2" ht="21" customHeight="1">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -4063,7 +4067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D343"/>
+  <dimension ref="A1:D365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10934,6 +10938,446 @@
         </is>
       </c>
     </row>
+    <row r="344" ht="21" customHeight="1">
+      <c r="A344" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B344" s="26" t="inlineStr">
+        <is>
+          <t>anb.australia</t>
+        </is>
+      </c>
+      <c r="C344" s="27" t="n">
+        <v>9734</v>
+      </c>
+      <c r="D344" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="345" ht="21" customHeight="1">
+      <c r="A345" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B345" s="26" t="inlineStr">
+        <is>
+          <t>cbrfitexpo</t>
+        </is>
+      </c>
+      <c r="C345" s="27" t="n">
+        <v>2220</v>
+      </c>
+      <c r="D345" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="21" customHeight="1">
+      <c r="A346" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B346" s="26" t="inlineStr">
+        <is>
+          <t>dfba_global</t>
+        </is>
+      </c>
+      <c r="C346" s="27" t="n">
+        <v>1837</v>
+      </c>
+      <c r="D346" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="21" customHeight="1">
+      <c r="A347" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B347" s="26" t="inlineStr">
+        <is>
+          <t>icn.indonesia</t>
+        </is>
+      </c>
+      <c r="C347" s="27" t="n">
+        <v>1838</v>
+      </c>
+      <c r="D347" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="348" ht="21" customHeight="1">
+      <c r="A348" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B348" s="26" t="inlineStr">
+        <is>
+          <t>icn_act</t>
+        </is>
+      </c>
+      <c r="C348" s="27" t="n">
+        <v>4591</v>
+      </c>
+      <c r="D348" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="349" ht="21" customHeight="1">
+      <c r="A349" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B349" s="26" t="inlineStr">
+        <is>
+          <t>icn_nsw</t>
+        </is>
+      </c>
+      <c r="C349" s="27" t="n">
+        <v>16036</v>
+      </c>
+      <c r="D349" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="350" ht="21" customHeight="1">
+      <c r="A350" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B350" s="26" t="inlineStr">
+        <is>
+          <t>icn_nt</t>
+        </is>
+      </c>
+      <c r="C350" s="27" t="n">
+        <v>1432</v>
+      </c>
+      <c r="D350" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="351" ht="21" customHeight="1">
+      <c r="A351" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B351" s="26" t="inlineStr">
+        <is>
+          <t>icn_sa</t>
+        </is>
+      </c>
+      <c r="C351" s="27" t="n">
+        <v>6716</v>
+      </c>
+      <c r="D351" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="352" ht="21" customHeight="1">
+      <c r="A352" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B352" s="26" t="inlineStr">
+        <is>
+          <t>icn_tasmania</t>
+        </is>
+      </c>
+      <c r="C352" s="27" t="n">
+        <v>2277</v>
+      </c>
+      <c r="D352" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="353" ht="21" customHeight="1">
+      <c r="A353" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B353" s="26" t="inlineStr">
+        <is>
+          <t>icn_victoria</t>
+        </is>
+      </c>
+      <c r="C353" s="27" t="n">
+        <v>12893</v>
+      </c>
+      <c r="D353" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="354" ht="21" customHeight="1">
+      <c r="A354" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B354" s="26" t="inlineStr">
+        <is>
+          <t>icn_wa</t>
+        </is>
+      </c>
+      <c r="C354" s="27" t="n">
+        <v>10997</v>
+      </c>
+      <c r="D354" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="355" ht="21" customHeight="1">
+      <c r="A355" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B355" s="26" t="inlineStr">
+        <is>
+          <t>icnnewzealand</t>
+        </is>
+      </c>
+      <c r="C355" s="27" t="n">
+        <v>6517</v>
+      </c>
+      <c r="D355" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="356" ht="21" customHeight="1">
+      <c r="A356" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B356" s="26" t="inlineStr">
+        <is>
+          <t>icnqld</t>
+        </is>
+      </c>
+      <c r="C356" s="27" t="n">
+        <v>17835</v>
+      </c>
+      <c r="D356" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="357" ht="21" customHeight="1">
+      <c r="A357" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B357" s="26" t="inlineStr">
+        <is>
+          <t>ifbbproleagueoz</t>
+        </is>
+      </c>
+      <c r="C357" s="27" t="n">
+        <v>57539</v>
+      </c>
+      <c r="D357" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="358" ht="21" customHeight="1">
+      <c r="A358" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B358" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia</t>
+        </is>
+      </c>
+      <c r="C358" s="27" t="n">
+        <v>15466</v>
+      </c>
+      <c r="D358" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="359" ht="21" customHeight="1">
+      <c r="A359" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B359" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_perth</t>
+        </is>
+      </c>
+      <c r="C359" s="27" t="n">
+        <v>1442</v>
+      </c>
+      <c r="D359" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="360" ht="21" customHeight="1">
+      <c r="A360" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B360" s="26" t="inlineStr">
+        <is>
+          <t>msfitnessaustralia_vic</t>
+        </is>
+      </c>
+      <c r="C360" s="27" t="n">
+        <v>935</v>
+      </c>
+      <c r="D360" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="361" ht="21" customHeight="1">
+      <c r="A361" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B361" s="26" t="inlineStr">
+        <is>
+          <t>nabbaaustralia</t>
+        </is>
+      </c>
+      <c r="C361" s="27" t="n">
+        <v>15721</v>
+      </c>
+      <c r="D361" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="362" ht="21" customHeight="1">
+      <c r="A362" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B362" s="26" t="inlineStr">
+        <is>
+          <t>nbaaustralia_official</t>
+        </is>
+      </c>
+      <c r="C362" s="27" t="n">
+        <v>18425</v>
+      </c>
+      <c r="D362" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="363" ht="21" customHeight="1">
+      <c r="A363" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B363" s="26" t="inlineStr">
+        <is>
+          <t>pca_australia</t>
+        </is>
+      </c>
+      <c r="C363" s="27" t="n">
+        <v>11413</v>
+      </c>
+      <c r="D363" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="364" ht="21" customHeight="1">
+      <c r="A364" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B364" s="26" t="inlineStr">
+        <is>
+          <t>wnbfaustralia</t>
+        </is>
+      </c>
+      <c r="C364" s="27" t="n">
+        <v>7252</v>
+      </c>
+      <c r="D364" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
+    <row r="365" ht="21" customHeight="1">
+      <c r="A365" s="26" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B365" s="26" t="inlineStr">
+        <is>
+          <t>ynf_australia</t>
+        </is>
+      </c>
+      <c r="C365" s="27" t="n">
+        <v>4620</v>
+      </c>
+      <c r="D365" s="26" t="inlineStr">
+        <is>
+          <t>apify_instagram_scraper</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>